<commit_message>
updating some default values
</commit_message>
<xml_diff>
--- a/Cost model data structure.xlsx
+++ b/Cost model data structure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samst\OneDrive\Documents\Work\Projects\PMH web tool\Thailand\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B37D8D0-8633-4366-8B46-6845354987DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB785F5-A9DD-4298-A728-6B3853AA5593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0D2E9C17-1371-9741-AFE8-B54FBA3315B4}"/>
   </bookViews>
@@ -6761,7 +6761,7 @@
         <v>1009</v>
       </c>
       <c r="E89" s="20">
-        <v>4375</v>
+        <v>526</v>
       </c>
       <c r="F89" s="35" t="s">
         <v>10</v>
@@ -6799,7 +6799,7 @@
         <v>1010</v>
       </c>
       <c r="E90" s="20">
-        <v>0</v>
+        <v>445</v>
       </c>
       <c r="F90" s="35" t="s">
         <v>10</v>
@@ -6943,7 +6943,7 @@
         <v>1014</v>
       </c>
       <c r="E94" s="20">
-        <v>0</v>
+        <v>1193</v>
       </c>
       <c r="F94" s="35" t="s">
         <v>10</v>
@@ -22484,7 +22484,7 @@
       </c>
       <c r="D745" s="8">
         <f>D149*inputs!E89</f>
-        <v>135866707.15723985</v>
+        <v>16335060.106219009</v>
       </c>
       <c r="E745" s="7" t="str">
         <f t="shared" ca="1" si="11"/>
@@ -22503,7 +22503,7 @@
       </c>
       <c r="D746" s="8">
         <f>D150*inputs!E90</f>
-        <v>0</v>
+        <v>9518884.3226606343</v>
       </c>
       <c r="E746" s="7" t="str">
         <f t="shared" ca="1" si="11"/>
@@ -22579,7 +22579,7 @@
       </c>
       <c r="D750" s="8">
         <f>D155*inputs!E94</f>
-        <v>0</v>
+        <v>32626546.958244383</v>
       </c>
       <c r="E750" s="7" t="str">
         <f t="shared" ca="1" si="11"/>
@@ -28283,7 +28283,7 @@
       </c>
       <c r="E41" s="11">
         <f>SUM(computations!D745:D751)</f>
-        <v>135866707.15723985</v>
+        <v>58480491.387124024</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.3">
@@ -28313,7 +28313,7 @@
       </c>
       <c r="E43" s="11">
         <f>E24+E36+E41</f>
-        <v>1071166797.2689085</v>
+        <v>993780581.49879265</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.3">
@@ -28343,7 +28343,7 @@
       </c>
       <c r="E45">
         <f>E43/1000000000</f>
-        <v>1.0711667972689085</v>
+        <v>0.99378058149879267</v>
       </c>
     </row>
     <row r="56" spans="2:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
slight edits to underlying spreadsheet
</commit_message>
<xml_diff>
--- a/Cost model data structure.xlsx
+++ b/Cost model data structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samst\OneDrive\Documents\Work\Projects\PMH web tool\Thailand\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9CE8CD-88A6-4FA8-B5EC-259DA47D8C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4B6F5B-EE2F-4A4D-93B1-4245BDBED76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{0D2E9C17-1371-9741-AFE8-B54FBA3315B4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{0D2E9C17-1371-9741-AFE8-B54FBA3315B4}"/>
   </bookViews>
   <sheets>
     <sheet name="inputs" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3495" uniqueCount="1054">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3497" uniqueCount="1056">
   <si>
     <t>Section</t>
   </si>
@@ -3299,6 +3299,12 @@
   </si>
   <si>
     <t>Valuing healthcare age 0-1, in USD</t>
+  </si>
+  <si>
+    <t>Mother's DALY</t>
+  </si>
+  <si>
+    <t>Mother's Income loss</t>
   </si>
 </sst>
 </file>
@@ -3387,7 +3393,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3430,6 +3436,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -3444,7 +3456,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3487,6 +3499,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4172,8 +4189,8 @@
       <c r="D10" s="12" t="s">
         <v>811</v>
       </c>
-      <c r="E10" s="25">
-        <v>0.04</v>
+      <c r="E10" s="23">
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="F10" s="35" t="s">
         <v>10</v>
@@ -4517,23 +4534,25 @@
       <c r="C21" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="38" t="s">
         <v>241</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="39">
         <f>1-E18</f>
         <v>0.60399999999999998</v>
       </c>
-      <c r="F21" s="34" t="s">
+      <c r="F21" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="I21" s="14" t="s">
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="J21" s="12" t="s">
+      <c r="J21" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="K21" s="12" t="s">
+      <c r="K21" s="38" t="s">
         <v>241</v>
       </c>
       <c r="L21" s="12" t="s">
@@ -4547,23 +4566,25 @@
       <c r="C22" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="38" t="s">
         <v>242</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="39">
         <f>1-E19</f>
         <v>0.34199999999999997</v>
       </c>
-      <c r="F22" s="34" t="s">
+      <c r="F22" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="I22" s="14" t="s">
+      <c r="G22" s="40"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="J22" s="12" t="s">
+      <c r="J22" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="K22" s="12" t="s">
+      <c r="K22" s="38" t="s">
         <v>242</v>
       </c>
       <c r="L22" s="12" t="s">
@@ -4577,23 +4598,25 @@
       <c r="C23" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="38" t="s">
         <v>247</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="39">
         <f>1-E22</f>
         <v>0.65800000000000003</v>
       </c>
-      <c r="F23" s="34" t="s">
+      <c r="F23" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="I23" s="14" t="s">
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="J23" s="12" t="s">
+      <c r="J23" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="K23" s="12" t="s">
+      <c r="K23" s="38" t="s">
         <v>247</v>
       </c>
       <c r="L23" s="12" t="s">
@@ -6440,15 +6463,17 @@
       <c r="C79" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D79" s="12" t="s">
+      <c r="D79" s="38" t="s">
         <v>277</v>
       </c>
-      <c r="E79" s="15">
-        <v>0</v>
-      </c>
-      <c r="F79" s="35" t="s">
+      <c r="E79" s="39">
+        <v>0</v>
+      </c>
+      <c r="F79" s="38" t="s">
         <v>9</v>
       </c>
+      <c r="G79" s="40"/>
+      <c r="H79" s="40"/>
       <c r="I79" s="14" t="s">
         <v>28</v>
       </c>
@@ -6472,16 +6497,18 @@
       <c r="C80" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D80" s="12" t="s">
+      <c r="D80" s="38" t="s">
         <v>487</v>
       </c>
-      <c r="E80" s="15">
+      <c r="E80" s="39">
         <f>(1-E73)</f>
         <v>0.96399999999999997</v>
       </c>
-      <c r="F80" s="35" t="s">
+      <c r="F80" s="38" t="s">
         <v>9</v>
       </c>
+      <c r="G80" s="40"/>
+      <c r="H80" s="40"/>
       <c r="I80" s="14" t="s">
         <v>28</v>
       </c>
@@ -6502,16 +6529,18 @@
       <c r="C81" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D81" s="12" t="s">
+      <c r="D81" s="38" t="s">
         <v>488</v>
       </c>
-      <c r="E81" s="15">
+      <c r="E81" s="39">
         <f>(1-E74)</f>
         <v>0.86699999999999999</v>
       </c>
-      <c r="F81" s="35" t="s">
+      <c r="F81" s="38" t="s">
         <v>9</v>
       </c>
+      <c r="G81" s="40"/>
+      <c r="H81" s="40"/>
       <c r="I81" s="14" t="s">
         <v>28</v>
       </c>
@@ -6532,16 +6561,18 @@
       <c r="C82" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D82" s="12" t="s">
+      <c r="D82" s="38" t="s">
         <v>489</v>
       </c>
-      <c r="E82" s="15">
+      <c r="E82" s="39">
         <f>(1-E75)</f>
         <v>0.872</v>
       </c>
-      <c r="F82" s="35" t="s">
+      <c r="F82" s="38" t="s">
         <v>9</v>
       </c>
+      <c r="G82" s="40"/>
+      <c r="H82" s="40"/>
       <c r="I82" s="14" t="s">
         <v>28</v>
       </c>
@@ -6562,16 +6593,18 @@
       <c r="C83" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D83" s="12" t="s">
+      <c r="D83" s="38" t="s">
         <v>490</v>
       </c>
-      <c r="E83" s="15">
+      <c r="E83" s="39">
         <f>(1-E76)</f>
         <v>0.75900000000000001</v>
       </c>
-      <c r="F83" s="35" t="s">
+      <c r="F83" s="38" t="s">
         <v>9</v>
       </c>
+      <c r="G83" s="40"/>
+      <c r="H83" s="40"/>
       <c r="I83" s="14" t="s">
         <v>28</v>
       </c>
@@ -6592,16 +6625,18 @@
       <c r="C84" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D84" s="12" t="s">
+      <c r="D84" s="38" t="s">
         <v>491</v>
       </c>
-      <c r="E84" s="15">
+      <c r="E84" s="39">
         <f t="shared" ref="E84:E85" si="0">(1-E77)</f>
         <v>0.95499999999999996</v>
       </c>
-      <c r="F84" s="35" t="s">
+      <c r="F84" s="38" t="s">
         <v>9</v>
       </c>
+      <c r="G84" s="40"/>
+      <c r="H84" s="40"/>
       <c r="I84" s="14" t="s">
         <v>28</v>
       </c>
@@ -6622,16 +6657,18 @@
       <c r="C85" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="D85" s="12" t="s">
+      <c r="D85" s="38" t="s">
         <v>492</v>
       </c>
-      <c r="E85" s="15">
+      <c r="E85" s="39">
         <f t="shared" si="0"/>
         <v>0.73499999999999999</v>
       </c>
-      <c r="F85" s="35" t="s">
+      <c r="F85" s="38" t="s">
         <v>9</v>
       </c>
+      <c r="G85" s="40"/>
+      <c r="H85" s="40"/>
       <c r="I85" s="14" t="s">
         <v>28</v>
       </c>
@@ -8916,7 +8953,7 @@
       </c>
       <c r="D38" s="28">
         <f>D2*inputs!E10</f>
-        <v>25911.976709165745</v>
+        <v>22672.979620520029</v>
       </c>
       <c r="E38" s="27" t="str">
         <f t="shared" ca="1" si="0"/>
@@ -9619,7 +9656,7 @@
       </c>
       <c r="D75" s="28">
         <f>D38*inputs!E17*inputs!E20</f>
-        <v>861.57322557976102</v>
+        <v>753.87657238229099</v>
       </c>
       <c r="E75" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -10322,7 +10359,7 @@
       </c>
       <c r="D112" s="28">
         <f>D75*(inputs!$E$26*inputs!$E$27)</f>
-        <v>3089601.5869290228</v>
+        <v>2703401.3885628954</v>
       </c>
       <c r="E112" s="27" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -10797,7 +10834,7 @@
       </c>
       <c r="D137" s="28">
         <f>D38*inputs!E29</f>
-        <v>57446852.364220455</v>
+        <v>50265995.818692908</v>
       </c>
       <c r="E137" s="27" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -27770,7 +27807,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE09E027-07AB-5B4E-B150-E88615AE26EE}">
-  <dimension ref="B2:F56"/>
+  <dimension ref="B2:G56"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="33.5" customWidth="1"/>
@@ -27836,7 +27873,7 @@
       </c>
       <c r="E6" s="11">
         <f>SUM(computations!D75:D87)</f>
-        <v>10750.131398313768</v>
+        <v>10642.434745116298</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
@@ -27851,7 +27888,7 @@
       </c>
       <c r="E7" s="11">
         <f>SUM(computations!D112:D123)</f>
-        <v>23250301.626918249</v>
+        <v>22864101.428552121</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
@@ -27911,7 +27948,7 @@
       </c>
       <c r="E11" s="11">
         <f>SUM(computations!D137:D148)</f>
-        <v>255298395.31782839</v>
+        <v>248117538.77230087</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -27977,7 +28014,7 @@
       </c>
       <c r="E16" s="11"/>
     </row>
-    <row r="17" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>770</v>
       </c>
@@ -27989,7 +28026,7 @@
       </c>
       <c r="E17" s="11"/>
     </row>
-    <row r="18" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>770</v>
       </c>
@@ -28001,7 +28038,7 @@
       </c>
       <c r="E18" s="11"/>
     </row>
-    <row r="19" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>770</v>
       </c>
@@ -28013,7 +28050,7 @@
       </c>
       <c r="E19" s="11"/>
     </row>
-    <row r="20" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>770</v>
       </c>
@@ -28025,7 +28062,7 @@
       </c>
       <c r="E20" s="11"/>
     </row>
-    <row r="21" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>770</v>
       </c>
@@ -28037,7 +28074,7 @@
       </c>
       <c r="E21" s="11"/>
     </row>
-    <row r="22" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>770</v>
       </c>
@@ -28049,7 +28086,7 @@
       </c>
       <c r="E22" s="11"/>
     </row>
-    <row r="23" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>770</v>
       </c>
@@ -28061,7 +28098,7 @@
       </c>
       <c r="E23" s="11"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>771</v>
       </c>
@@ -28075,8 +28112,11 @@
         <f>SUM(computations!D500:D644)</f>
         <v>663958226.35652614</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G24" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>771</v>
       </c>
@@ -28088,7 +28128,7 @@
       </c>
       <c r="E25" s="11"/>
     </row>
-    <row r="26" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>771</v>
       </c>
@@ -28100,7 +28140,7 @@
       </c>
       <c r="E26" s="11"/>
     </row>
-    <row r="27" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>771</v>
       </c>
@@ -28112,7 +28152,7 @@
       </c>
       <c r="E27" s="11"/>
     </row>
-    <row r="28" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>771</v>
       </c>
@@ -28124,7 +28164,7 @@
       </c>
       <c r="E28" s="11"/>
     </row>
-    <row r="29" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>771</v>
       </c>
@@ -28136,7 +28176,7 @@
       </c>
       <c r="E29" s="11"/>
     </row>
-    <row r="30" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>771</v>
       </c>
@@ -28148,7 +28188,7 @@
       </c>
       <c r="E30" s="11"/>
     </row>
-    <row r="31" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>771</v>
       </c>
@@ -28160,7 +28200,7 @@
       </c>
       <c r="E31" s="11"/>
     </row>
-    <row r="32" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>771</v>
       </c>
@@ -28172,7 +28212,7 @@
       </c>
       <c r="E32" s="11"/>
     </row>
-    <row r="33" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>771</v>
       </c>
@@ -28184,7 +28224,7 @@
       </c>
       <c r="E33" s="11"/>
     </row>
-    <row r="34" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>771</v>
       </c>
@@ -28196,7 +28236,7 @@
       </c>
       <c r="E34" s="11"/>
     </row>
-    <row r="35" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>771</v>
       </c>
@@ -28208,7 +28248,7 @@
       </c>
       <c r="E35" s="11"/>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>772</v>
       </c>
@@ -28222,8 +28262,12 @@
         <f>SUM(computations!D645:D744)</f>
         <v>270504021.46303487</v>
       </c>
-    </row>
-    <row r="37" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G36" s="11">
+        <f>E7+E5+E9</f>
+        <v>226186346.58814651</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>772</v>
       </c>
@@ -28235,7 +28279,7 @@
       </c>
       <c r="E37" s="11"/>
     </row>
-    <row r="38" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>772</v>
       </c>
@@ -28247,7 +28291,7 @@
       </c>
       <c r="E38" s="11"/>
     </row>
-    <row r="39" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>772</v>
       </c>
@@ -28259,7 +28303,7 @@
       </c>
       <c r="E39" s="11"/>
     </row>
-    <row r="40" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>772</v>
       </c>
@@ -28271,7 +28315,7 @@
       </c>
       <c r="E40" s="11"/>
     </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>758</v>
       </c>
@@ -28285,8 +28329,11 @@
         <f>SUM(computations!D745:D751)</f>
         <v>58438963.115779579</v>
       </c>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="G41" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>774</v>
       </c>
@@ -28296,12 +28343,16 @@
       <c r="D42" t="s">
         <v>774</v>
       </c>
-      <c r="E42" s="11">
-        <f>E5+E6+E7+E9+E10+E11</f>
-        <v>1165171053.4243438</v>
-      </c>
-    </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="E42" s="41">
+        <f>E5+E7+E9+E10+E11</f>
+        <v>1157593246.549052</v>
+      </c>
+      <c r="G42" s="11">
+        <f>E10+E11</f>
+        <v>931406899.96090531</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>773</v>
       </c>
@@ -28316,7 +28367,7 @@
         <v>992901210.93534064</v>
       </c>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>774</v>
       </c>
@@ -28326,12 +28377,12 @@
       <c r="D44" t="s">
         <v>804</v>
       </c>
-      <c r="E44">
+      <c r="E44" s="42">
         <f>E42/1000000000</f>
-        <v>1.1651710534243438</v>
-      </c>
-    </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.3">
+        <v>1.1575932465490519</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>773</v>
       </c>
@@ -28352,7 +28403,7 @@
       </c>
       <c r="E56" s="11">
         <f>SUM(E5+E7+E9)/1000000</f>
-        <v>226.57254678651267</v>
+        <v>226.18634658814651</v>
       </c>
       <c r="F56" t="s">
         <v>823</v>

</xml_diff>